<commit_message>
Baja de 10 asesores, crédito a asesor 2 interno, acumulado cuatrimestral de leads
</commit_message>
<xml_diff>
--- a/data/APARTADO.xlsx
+++ b/data/APARTADO.xlsx
@@ -21763,1638 +21763,420 @@
       </c>
     </row>
     <row r="167" ht="22.5" customHeight="1" s="52">
-      <c r="A167" s="53" t="n"/>
+      <c r="A167" s="49" t="n"/>
       <c r="B167" s="50" t="n"/>
-      <c r="C167" s="50" t="n">
-        <v>1900000</v>
-      </c>
-      <c r="D167" s="31" t="inlineStr">
-        <is>
-          <t>VENTA</t>
-        </is>
-      </c>
-      <c r="E167" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
-      <c r="F167" s="35" t="inlineStr">
-        <is>
-          <t>EB-UL0622</t>
-        </is>
-      </c>
-      <c r="G167" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="H167" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I167" s="50" t="inlineStr">
-        <is>
-          <t>Marisol Huerta Ruiz</t>
-        </is>
-      </c>
-      <c r="J167" s="50" t="inlineStr">
-        <is>
-          <t>Recomendado</t>
-        </is>
-      </c>
-      <c r="K167" s="50" t="inlineStr">
-        <is>
-          <t>PAGADO</t>
-        </is>
-      </c>
-      <c r="L167" s="50" t="inlineStr">
-        <is>
-          <t>Erik Trotter Bustamante Remax Terra</t>
-        </is>
-      </c>
-      <c r="M167" s="50" t="n">
-        <v>4422580793</v>
-      </c>
-      <c r="N167" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O167" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P167" s="50" t="inlineStr">
-        <is>
-          <t>Elsa morales Franco</t>
-        </is>
-      </c>
-      <c r="Q167" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R167" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S167" s="50" t="inlineStr">
-        <is>
-          <t>COMPARTIDA</t>
-        </is>
-      </c>
-      <c r="T167" s="51" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="U167" s="50" t="n">
-        <v>95000</v>
-      </c>
-      <c r="V167" s="50" t="n">
-        <v>95000</v>
-      </c>
-      <c r="W167" s="35" t="inlineStr">
-        <is>
-          <t>Cumbres del lago 45 Juriquilla, Querétaro</t>
-        </is>
-      </c>
-      <c r="X167" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y167" s="50" t="n">
-        <v>19000</v>
-      </c>
-      <c r="Z167" s="50" t="inlineStr">
-        <is>
-          <t>CERRADA</t>
-        </is>
-      </c>
-      <c r="AA167" s="53" t="n">
-        <v>46036</v>
-      </c>
-      <c r="AB167" s="53" t="n">
-        <v>46066</v>
-      </c>
-      <c r="AC167" s="31" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AD167" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
+      <c r="C167" s="50" t="n"/>
+      <c r="D167" s="50" t="n"/>
+      <c r="E167" s="50" t="n"/>
+      <c r="F167" s="35" t="n"/>
+      <c r="G167" s="50" t="n"/>
+      <c r="H167" s="42" t="n"/>
+      <c r="I167" s="50" t="n"/>
+      <c r="J167" s="50" t="n"/>
+      <c r="K167" s="50" t="n"/>
+      <c r="L167" s="50" t="n"/>
+      <c r="M167" s="50" t="n"/>
+      <c r="N167" s="50" t="n"/>
+      <c r="O167" s="50" t="n"/>
+      <c r="P167" s="50" t="n"/>
+      <c r="Q167" s="50" t="n"/>
+      <c r="R167" s="50" t="n"/>
+      <c r="S167" s="50" t="n"/>
+      <c r="T167" s="51" t="n"/>
+      <c r="U167" s="50" t="n"/>
+      <c r="V167" s="50" t="n"/>
+      <c r="W167" s="35" t="n"/>
+      <c r="X167" s="50" t="n"/>
+      <c r="Y167" s="50" t="n"/>
+      <c r="Z167" s="50" t="n"/>
+      <c r="AA167" s="39" t="n"/>
+      <c r="AB167" s="39" t="n"/>
+      <c r="AC167" s="42" t="n"/>
+      <c r="AD167" s="50" t="n"/>
     </row>
     <row r="168" ht="22.5" customHeight="1" s="52">
-      <c r="A168" s="53" t="n"/>
+      <c r="A168" s="49" t="n"/>
       <c r="B168" s="50" t="n"/>
-      <c r="C168" s="50" t="n">
-        <v>23000</v>
-      </c>
-      <c r="D168" s="31" t="inlineStr">
-        <is>
-          <t>RENTA</t>
-        </is>
-      </c>
-      <c r="E168" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
-      <c r="F168" s="35" t="inlineStr">
-        <is>
-          <t>RDR663936-495</t>
-        </is>
-      </c>
-      <c r="G168" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="H168" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I168" s="50" t="inlineStr">
-        <is>
-          <t>Nidia Gisela García Trujillo</t>
-        </is>
-      </c>
-      <c r="J168" s="50" t="inlineStr">
-        <is>
-          <t>Guardia</t>
-        </is>
-      </c>
-      <c r="K168" s="50" t="inlineStr">
-        <is>
-          <t>PAGADO</t>
-        </is>
-      </c>
-      <c r="L168" s="50" t="inlineStr">
-        <is>
-          <t>Lorena Payan Remax Terra</t>
-        </is>
-      </c>
-      <c r="M168" s="50" t="inlineStr">
-        <is>
-          <t>442 803 1452</t>
-        </is>
-      </c>
-      <c r="N168" s="50" t="inlineStr">
-        <is>
-          <t>ERIHK ENRIQUE GARRIDO ALBARRAN</t>
-        </is>
-      </c>
-      <c r="O168" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P168" s="50" t="inlineStr">
-        <is>
-          <t>Hector Alexandro Hidalgo Mungaray</t>
-        </is>
-      </c>
-      <c r="Q168" s="50" t="n">
-        <v>6622446008</v>
-      </c>
-      <c r="R168" s="50" t="inlineStr">
-        <is>
-          <t>hidalgomungaray@gmail.com</t>
-        </is>
-      </c>
-      <c r="S168" s="50" t="inlineStr">
-        <is>
-          <t>COMPARTIDA</t>
-        </is>
-      </c>
-      <c r="T168" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="U168" s="50" t="n">
-        <v>23000</v>
-      </c>
-      <c r="V168" s="50" t="n">
-        <v>23000</v>
-      </c>
-      <c r="W168" s="35" t="inlineStr">
-        <is>
-          <t>Camino Real de Carretas No 300 8 Milenio III, Querétaro, Querétaro</t>
-        </is>
-      </c>
-      <c r="X168" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y168" s="50" t="n">
-        <v>5750</v>
-      </c>
-      <c r="Z168" s="50" t="inlineStr">
-        <is>
-          <t>CERRADA</t>
-        </is>
-      </c>
-      <c r="AA168" s="53" t="n">
-        <v>46044</v>
-      </c>
-      <c r="AB168" s="53" t="n">
-        <v>46051</v>
-      </c>
-      <c r="AC168" s="31" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AD168" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
+      <c r="C168" s="50" t="n"/>
+      <c r="D168" s="50" t="n"/>
+      <c r="E168" s="50" t="n"/>
+      <c r="F168" s="35" t="n"/>
+      <c r="G168" s="50" t="n"/>
+      <c r="H168" s="42" t="n"/>
+      <c r="I168" s="50" t="n"/>
+      <c r="J168" s="50" t="n"/>
+      <c r="K168" s="50" t="n"/>
+      <c r="L168" s="50" t="n"/>
+      <c r="M168" s="50" t="n"/>
+      <c r="N168" s="50" t="n"/>
+      <c r="O168" s="50" t="n"/>
+      <c r="P168" s="50" t="n"/>
+      <c r="Q168" s="50" t="n"/>
+      <c r="R168" s="50" t="n"/>
+      <c r="S168" s="50" t="n"/>
+      <c r="T168" s="51" t="n"/>
+      <c r="U168" s="50" t="n"/>
+      <c r="V168" s="50" t="n"/>
+      <c r="W168" s="35" t="n"/>
+      <c r="X168" s="50" t="n"/>
+      <c r="Y168" s="50" t="n"/>
+      <c r="Z168" s="50" t="n"/>
+      <c r="AA168" s="39" t="n"/>
+      <c r="AB168" s="39" t="n"/>
+      <c r="AC168" s="42" t="n"/>
+      <c r="AD168" s="50" t="n"/>
     </row>
     <row r="169" ht="22.5" customHeight="1" s="52">
-      <c r="A169" s="53" t="n"/>
+      <c r="A169" s="49" t="n"/>
       <c r="B169" s="50" t="n"/>
-      <c r="C169" s="50" t="n">
-        <v>20000</v>
-      </c>
-      <c r="D169" s="31" t="inlineStr">
-        <is>
-          <t>RENTA</t>
-        </is>
-      </c>
-      <c r="E169" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
-      <c r="F169" s="35" t="inlineStr">
-        <is>
-          <t>RCV621951-495</t>
-        </is>
-      </c>
-      <c r="G169" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="H169" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I169" s="50" t="inlineStr">
-        <is>
-          <t>María de los Ángeles Bostal</t>
-        </is>
-      </c>
-      <c r="J169" s="50" t="inlineStr">
-        <is>
-          <t>Re/Max</t>
-        </is>
-      </c>
-      <c r="K169" s="50" t="inlineStr">
-        <is>
-          <t>PAGADO</t>
-        </is>
-      </c>
-      <c r="L169" s="50" t="inlineStr">
-        <is>
-          <t>Alma Verónica Flores Guzmán Remax Terra</t>
-        </is>
-      </c>
-      <c r="M169" s="50" t="inlineStr">
-        <is>
-          <t>55 5102 6906</t>
-        </is>
-      </c>
-      <c r="N169" s="50" t="inlineStr">
-        <is>
-          <t>Martin Uehara Argentino</t>
-        </is>
-      </c>
-      <c r="O169" s="50" t="inlineStr">
-        <is>
-          <t>442 226 0673</t>
-        </is>
-      </c>
-      <c r="P169" s="50" t="inlineStr">
-        <is>
-          <t>Rosangela</t>
-        </is>
-      </c>
-      <c r="Q169" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R169" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S169" s="50" t="inlineStr">
-        <is>
-          <t>COMPARTIDA</t>
-        </is>
-      </c>
-      <c r="T169" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="U169" s="50" t="n">
-        <v>25000</v>
-      </c>
-      <c r="V169" s="50" t="n">
-        <v>25000</v>
-      </c>
-      <c r="W169" s="35" t="inlineStr">
-        <is>
-          <t>Sendero de la Alegria 3 Milenio III, Querétaro, Querétaro</t>
-        </is>
-      </c>
-      <c r="X169" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y169" s="50" t="n">
-        <v>6250</v>
-      </c>
-      <c r="Z169" s="50" t="inlineStr">
-        <is>
-          <t>CERRADA</t>
-        </is>
-      </c>
-      <c r="AA169" s="53" t="n">
-        <v>46051</v>
-      </c>
-      <c r="AB169" s="53" t="n">
-        <v>46069</v>
-      </c>
-      <c r="AC169" s="31" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AD169" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
+      <c r="C169" s="50" t="n"/>
+      <c r="D169" s="50" t="n"/>
+      <c r="E169" s="50" t="n"/>
+      <c r="F169" s="35" t="n"/>
+      <c r="G169" s="50" t="n"/>
+      <c r="H169" s="42" t="n"/>
+      <c r="I169" s="50" t="n"/>
+      <c r="J169" s="50" t="n"/>
+      <c r="K169" s="50" t="n"/>
+      <c r="L169" s="50" t="n"/>
+      <c r="M169" s="50" t="n"/>
+      <c r="N169" s="50" t="n"/>
+      <c r="O169" s="50" t="n"/>
+      <c r="P169" s="50" t="n"/>
+      <c r="Q169" s="50" t="n"/>
+      <c r="R169" s="50" t="n"/>
+      <c r="S169" s="50" t="n"/>
+      <c r="T169" s="51" t="n"/>
+      <c r="U169" s="50" t="n"/>
+      <c r="V169" s="50" t="n"/>
+      <c r="W169" s="35" t="n"/>
+      <c r="X169" s="50" t="n"/>
+      <c r="Y169" s="50" t="n"/>
+      <c r="Z169" s="50" t="n"/>
+      <c r="AA169" s="39" t="n"/>
+      <c r="AB169" s="39" t="n"/>
+      <c r="AC169" s="42" t="n"/>
+      <c r="AD169" s="50" t="n"/>
     </row>
     <row r="170" ht="22.5" customHeight="1" s="52">
-      <c r="A170" s="53" t="n"/>
+      <c r="A170" s="49" t="n"/>
       <c r="B170" s="50" t="n"/>
-      <c r="C170" s="50" t="n">
-        <v>17500</v>
-      </c>
-      <c r="D170" s="31" t="inlineStr">
-        <is>
-          <t>RENTA</t>
-        </is>
-      </c>
-      <c r="E170" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
-      <c r="F170" s="35" t="inlineStr">
-        <is>
-          <t>CLR645464-495</t>
-        </is>
-      </c>
-      <c r="G170" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="H170" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I170" s="50" t="inlineStr">
-        <is>
-          <t>Alma Verónica Flores Guzmán</t>
-        </is>
-      </c>
-      <c r="J170" s="50" t="inlineStr">
-        <is>
-          <t>Guardia</t>
-        </is>
-      </c>
-      <c r="K170" s="50" t="inlineStr">
-        <is>
-          <t>PAGADO</t>
-        </is>
-      </c>
-      <c r="L170" s="50" t="inlineStr">
-        <is>
-          <t>Héctor de la Peña Remax Terra</t>
-        </is>
-      </c>
-      <c r="M170" s="50" t="inlineStr">
-        <is>
-          <t>442 475 2253</t>
-        </is>
-      </c>
-      <c r="N170" s="50" t="inlineStr">
-        <is>
-          <t>Martin Uehara Argentino</t>
-        </is>
-      </c>
-      <c r="O170" s="50" t="inlineStr">
-        <is>
-          <t>442-226-0673</t>
-        </is>
-      </c>
-      <c r="P170" s="50" t="inlineStr">
-        <is>
-          <t>María de los Ángeles Aguilera Mendoza</t>
-        </is>
-      </c>
-      <c r="Q170" s="50" t="inlineStr">
-        <is>
-          <t>871 158 4503</t>
-        </is>
-      </c>
-      <c r="R170" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S170" s="50" t="inlineStr">
-        <is>
-          <t>COMPARTIDA</t>
-        </is>
-      </c>
-      <c r="T170" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="U170" s="50" t="n">
-        <v>17500</v>
-      </c>
-      <c r="V170" s="50" t="n">
-        <v>17500</v>
-      </c>
-      <c r="W170" s="35" t="inlineStr">
-        <is>
-          <t>AVENIDA PEÑUELAS 19 13 FRACCIONAMIENTO INDUSTRIAL SAN PEDRITO PEÑUELAS, QUERÉTARO</t>
-        </is>
-      </c>
-      <c r="X170" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y170" s="50" t="n">
-        <v>4375</v>
-      </c>
-      <c r="Z170" s="50" t="inlineStr">
-        <is>
-          <t>CERRADA</t>
-        </is>
-      </c>
-      <c r="AA170" s="53" t="n">
-        <v>46066</v>
-      </c>
-      <c r="AB170" s="53" t="n">
-        <v>46070</v>
-      </c>
-      <c r="AC170" s="31" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AD170" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
+      <c r="C170" s="50" t="n"/>
+      <c r="D170" s="50" t="n"/>
+      <c r="E170" s="50" t="n"/>
+      <c r="F170" s="35" t="n"/>
+      <c r="G170" s="50" t="n"/>
+      <c r="H170" s="42" t="n"/>
+      <c r="I170" s="50" t="n"/>
+      <c r="J170" s="50" t="n"/>
+      <c r="K170" s="50" t="n"/>
+      <c r="L170" s="50" t="n"/>
+      <c r="M170" s="50" t="n"/>
+      <c r="N170" s="50" t="n"/>
+      <c r="O170" s="50" t="n"/>
+      <c r="P170" s="50" t="n"/>
+      <c r="Q170" s="50" t="n"/>
+      <c r="R170" s="50" t="n"/>
+      <c r="S170" s="50" t="n"/>
+      <c r="T170" s="51" t="n"/>
+      <c r="U170" s="50" t="n"/>
+      <c r="V170" s="50" t="n"/>
+      <c r="W170" s="35" t="n"/>
+      <c r="X170" s="50" t="n"/>
+      <c r="Y170" s="50" t="n"/>
+      <c r="Z170" s="50" t="n"/>
+      <c r="AA170" s="39" t="n"/>
+      <c r="AB170" s="39" t="n"/>
+      <c r="AC170" s="42" t="n"/>
+      <c r="AD170" s="50" t="n"/>
     </row>
     <row r="171" ht="22.5" customHeight="1" s="52">
-      <c r="A171" s="53" t="n"/>
+      <c r="A171" s="49" t="n"/>
       <c r="B171" s="50" t="n"/>
-      <c r="C171" s="50" t="n">
-        <v>2675325.09</v>
-      </c>
-      <c r="D171" s="31" t="inlineStr">
-        <is>
-          <t>VENTA</t>
-        </is>
-      </c>
-      <c r="E171" s="50" t="inlineStr">
-        <is>
-          <t>TRANSFERENCIA</t>
-        </is>
-      </c>
-      <c r="F171" s="35" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G171" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="H171" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I171" s="50" t="inlineStr">
-        <is>
-          <t>Consuelo Ramírez</t>
-        </is>
-      </c>
-      <c r="J171" s="50" t="inlineStr">
-        <is>
-          <t>Recomendado</t>
-        </is>
-      </c>
-      <c r="K171" s="50" t="inlineStr">
-        <is>
-          <t>PAGADO</t>
-        </is>
-      </c>
-      <c r="L171" s="50" t="inlineStr">
-        <is>
-          <t>Erik Trotter Bustamante Remax Terra</t>
-        </is>
-      </c>
-      <c r="M171" s="50" t="inlineStr">
-        <is>
-          <t>442 468 9256</t>
-        </is>
-      </c>
-      <c r="N171" s="50" t="inlineStr">
-        <is>
-          <t>Gabriela cantu estrada</t>
-        </is>
-      </c>
-      <c r="O171" s="50" t="n">
-        <v>4421865223</v>
-      </c>
-      <c r="P171" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q171" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R171" s="50" t="inlineStr">
-        <is>
-          <t>cantu_08@hotmail.com</t>
-        </is>
-      </c>
-      <c r="S171" s="50" t="inlineStr">
-        <is>
-          <t>COMPARTIDA</t>
-        </is>
-      </c>
-      <c r="T171" s="51" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="U171" s="50" t="n">
-        <v>80259.75</v>
-      </c>
-      <c r="V171" s="50" t="n">
-        <v>80259.75</v>
-      </c>
-      <c r="W171" s="35" t="inlineStr">
-        <is>
-          <t>Fracc zircon el Márquez valle de los olivos depa a102 900 El marqués, Querétaro</t>
-        </is>
-      </c>
-      <c r="X171" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y171" s="50" t="n">
-        <v>40129.88</v>
-      </c>
-      <c r="Z171" s="50" t="inlineStr">
-        <is>
-          <t>CERRADA</t>
-        </is>
-      </c>
-      <c r="AA171" s="53" t="n">
-        <v>46147</v>
-      </c>
-      <c r="AB171" s="53" t="n">
-        <v>46185</v>
-      </c>
-      <c r="AC171" s="31" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AD171" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
+      <c r="C171" s="50" t="n"/>
+      <c r="D171" s="50" t="n"/>
+      <c r="E171" s="50" t="n"/>
+      <c r="F171" s="35" t="n"/>
+      <c r="G171" s="50" t="n"/>
+      <c r="H171" s="42" t="n"/>
+      <c r="I171" s="50" t="n"/>
+      <c r="J171" s="50" t="n"/>
+      <c r="K171" s="50" t="n"/>
+      <c r="L171" s="50" t="n"/>
+      <c r="M171" s="50" t="n"/>
+      <c r="N171" s="50" t="n"/>
+      <c r="O171" s="50" t="n"/>
+      <c r="P171" s="50" t="n"/>
+      <c r="Q171" s="50" t="n"/>
+      <c r="R171" s="50" t="n"/>
+      <c r="S171" s="50" t="n"/>
+      <c r="T171" s="51" t="n"/>
+      <c r="U171" s="50" t="n"/>
+      <c r="V171" s="50" t="n"/>
+      <c r="W171" s="35" t="n"/>
+      <c r="X171" s="50" t="n"/>
+      <c r="Y171" s="50" t="n"/>
+      <c r="Z171" s="50" t="n"/>
+      <c r="AA171" s="39" t="n"/>
+      <c r="AB171" s="39" t="n"/>
+      <c r="AC171" s="42" t="n"/>
+      <c r="AD171" s="50" t="n"/>
     </row>
     <row r="172" ht="22.5" customHeight="1" s="52">
-      <c r="A172" s="53" t="n"/>
+      <c r="A172" s="49" t="n"/>
       <c r="B172" s="50" t="n"/>
-      <c r="C172" s="50" t="n">
-        <v>11500</v>
-      </c>
-      <c r="D172" s="31" t="inlineStr">
-        <is>
-          <t>RENTA</t>
-        </is>
-      </c>
-      <c r="E172" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
-      <c r="F172" s="35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RCR672284-495 </t>
-        </is>
-      </c>
-      <c r="G172" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="H172" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I172" s="50" t="inlineStr">
-        <is>
-          <t>Christian Alvarado Martínez</t>
-        </is>
-      </c>
-      <c r="J172" s="50" t="inlineStr">
-        <is>
-          <t>Guardia</t>
-        </is>
-      </c>
-      <c r="K172" s="50" t="inlineStr">
-        <is>
-          <t>PAGADO</t>
-        </is>
-      </c>
-      <c r="L172" s="50" t="inlineStr">
-        <is>
-          <t>María Elena Romano Pelayo Remax Terra</t>
-        </is>
-      </c>
-      <c r="M172" s="50" t="inlineStr">
-        <is>
-          <t>442 822 6699</t>
-        </is>
-      </c>
-      <c r="N172" s="50" t="inlineStr">
-        <is>
-          <t>María Lili Hiller Plazas</t>
-        </is>
-      </c>
-      <c r="O172" s="50" t="inlineStr">
-        <is>
-          <t>938 188 3659</t>
-        </is>
-      </c>
-      <c r="P172" s="50" t="inlineStr">
-        <is>
-          <t>Edith Osorio Chávez</t>
-        </is>
-      </c>
-      <c r="Q172" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R172" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S172" s="50" t="inlineStr">
-        <is>
-          <t>COMPARTIDA</t>
-        </is>
-      </c>
-      <c r="T172" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="U172" s="50" t="n">
-        <v>11500</v>
-      </c>
-      <c r="V172" s="50" t="n">
-        <v>11500</v>
-      </c>
-      <c r="W172" s="35" t="inlineStr">
-        <is>
-          <t>Cirrus 308 25, Privada Eriz, Real Solare, El Marqués Querétaro</t>
-        </is>
-      </c>
-      <c r="X172" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y172" s="50" t="n">
-        <v>2875</v>
-      </c>
-      <c r="Z172" s="50" t="inlineStr">
-        <is>
-          <t>CERRADA</t>
-        </is>
-      </c>
-      <c r="AA172" s="53" t="n">
-        <v>46135</v>
-      </c>
-      <c r="AB172" s="53" t="n">
-        <v>46146</v>
-      </c>
-      <c r="AC172" s="31" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AD172" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
+      <c r="C172" s="50" t="n"/>
+      <c r="D172" s="50" t="n"/>
+      <c r="E172" s="50" t="n"/>
+      <c r="F172" s="35" t="n"/>
+      <c r="G172" s="50" t="n"/>
+      <c r="H172" s="42" t="n"/>
+      <c r="I172" s="50" t="n"/>
+      <c r="J172" s="50" t="n"/>
+      <c r="K172" s="50" t="n"/>
+      <c r="L172" s="50" t="n"/>
+      <c r="M172" s="50" t="n"/>
+      <c r="N172" s="50" t="n"/>
+      <c r="O172" s="50" t="n"/>
+      <c r="P172" s="50" t="n"/>
+      <c r="Q172" s="50" t="n"/>
+      <c r="R172" s="50" t="n"/>
+      <c r="S172" s="50" t="n"/>
+      <c r="T172" s="51" t="n"/>
+      <c r="U172" s="50" t="n"/>
+      <c r="V172" s="50" t="n"/>
+      <c r="W172" s="35" t="n"/>
+      <c r="X172" s="50" t="n"/>
+      <c r="Y172" s="50" t="n"/>
+      <c r="Z172" s="50" t="n"/>
+      <c r="AA172" s="39" t="n"/>
+      <c r="AB172" s="39" t="n"/>
+      <c r="AC172" s="42" t="n"/>
+      <c r="AD172" s="50" t="n"/>
     </row>
     <row r="173" ht="22.5" customHeight="1" s="52">
-      <c r="A173" s="53" t="n"/>
+      <c r="A173" s="49" t="n"/>
       <c r="B173" s="50" t="n"/>
-      <c r="C173" s="50" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="D173" s="31" t="inlineStr">
-        <is>
-          <t>VENTA</t>
-        </is>
-      </c>
-      <c r="E173" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
-      <c r="F173" s="35" t="inlineStr">
-        <is>
-          <t>CLV648980-495</t>
-        </is>
-      </c>
-      <c r="G173" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="H173" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I173" s="50" t="inlineStr">
-        <is>
-          <t>Christian Alvarado Martínez</t>
-        </is>
-      </c>
-      <c r="J173" s="50" t="inlineStr">
-        <is>
-          <t>Guardia</t>
-        </is>
-      </c>
-      <c r="K173" s="50" t="inlineStr">
-        <is>
-          <t>PAGADO</t>
-        </is>
-      </c>
-      <c r="L173" s="50" t="inlineStr">
-        <is>
-          <t>Lorena Ramos Quevedo Remax Terra</t>
-        </is>
-      </c>
-      <c r="M173" s="50" t="n">
-        <v>4428226699</v>
-      </c>
-      <c r="N173" s="50" t="inlineStr">
-        <is>
-          <t>DAVID VAZQUEZ REA</t>
-        </is>
-      </c>
-      <c r="O173" s="50" t="n">
-        <v>4424614137</v>
-      </c>
-      <c r="P173" s="50" t="inlineStr">
-        <is>
-          <t>JOSE ADRIAN RUIZ GARDUÑO</t>
-        </is>
-      </c>
-      <c r="Q173" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R173" s="50" t="inlineStr">
-        <is>
-          <t>davisuf9@gmail.com</t>
-        </is>
-      </c>
-      <c r="S173" s="50" t="inlineStr">
-        <is>
-          <t>COMPARTIDA</t>
-        </is>
-      </c>
-      <c r="T173" s="51" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="U173" s="50" t="n">
-        <v>60000</v>
-      </c>
-      <c r="V173" s="50" t="n">
-        <v>60000</v>
-      </c>
-      <c r="W173" s="35" t="inlineStr">
-        <is>
-          <t>CALZADA DE BELEN 426 LOMAS DE SAN PEDRITO PEÑUELAS, QUERÉTARO</t>
-        </is>
-      </c>
-      <c r="X173" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y173" s="50" t="n">
-        <v>15000</v>
-      </c>
-      <c r="Z173" s="50" t="inlineStr">
-        <is>
-          <t>CERRADA</t>
-        </is>
-      </c>
-      <c r="AA173" s="53" t="n">
-        <v>46221</v>
-      </c>
-      <c r="AB173" s="53" t="n">
-        <v>46246</v>
-      </c>
-      <c r="AC173" s="31" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AD173" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
+      <c r="C173" s="50" t="n"/>
+      <c r="D173" s="50" t="n"/>
+      <c r="E173" s="50" t="n"/>
+      <c r="F173" s="35" t="n"/>
+      <c r="G173" s="50" t="n"/>
+      <c r="H173" s="42" t="n"/>
+      <c r="I173" s="50" t="n"/>
+      <c r="J173" s="50" t="n"/>
+      <c r="K173" s="50" t="n"/>
+      <c r="L173" s="50" t="n"/>
+      <c r="M173" s="50" t="n"/>
+      <c r="N173" s="50" t="n"/>
+      <c r="O173" s="50" t="n"/>
+      <c r="P173" s="50" t="n"/>
+      <c r="Q173" s="50" t="n"/>
+      <c r="R173" s="50" t="n"/>
+      <c r="S173" s="50" t="n"/>
+      <c r="T173" s="51" t="n"/>
+      <c r="U173" s="50" t="n"/>
+      <c r="V173" s="50" t="n"/>
+      <c r="W173" s="35" t="n"/>
+      <c r="X173" s="50" t="n"/>
+      <c r="Y173" s="50" t="n"/>
+      <c r="Z173" s="50" t="n"/>
+      <c r="AA173" s="39" t="n"/>
+      <c r="AB173" s="39" t="n"/>
+      <c r="AC173" s="42" t="n"/>
+      <c r="AD173" s="50" t="n"/>
     </row>
     <row r="174" ht="22.5" customHeight="1" s="52">
-      <c r="A174" s="53" t="n"/>
+      <c r="A174" s="49" t="n"/>
       <c r="B174" s="50" t="n"/>
-      <c r="C174" s="50" t="n">
-        <v>22500</v>
-      </c>
-      <c r="D174" s="31" t="inlineStr">
-        <is>
-          <t>RENTA</t>
-        </is>
-      </c>
-      <c r="E174" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
-      <c r="F174" s="35" t="inlineStr">
-        <is>
-          <t>RCR681291-495</t>
-        </is>
-      </c>
-      <c r="G174" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="H174" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I174" s="50" t="inlineStr">
-        <is>
-          <t>María de los Ángeles Bostal</t>
-        </is>
-      </c>
-      <c r="J174" s="50" t="inlineStr">
-        <is>
-          <t>Guardia</t>
-        </is>
-      </c>
-      <c r="K174" s="50" t="inlineStr">
-        <is>
-          <t>PAGADO</t>
-        </is>
-      </c>
-      <c r="L174" s="50" t="inlineStr">
-        <is>
-          <t>Adriana Calva Remax Terra</t>
-        </is>
-      </c>
-      <c r="M174" s="50" t="inlineStr">
-        <is>
-          <t>55 5102 6906</t>
-        </is>
-      </c>
-      <c r="N174" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O174" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P174" s="50" t="inlineStr">
-        <is>
-          <t>José Martín Fernandéz Jasso / Ericka García</t>
-        </is>
-      </c>
-      <c r="Q174" s="50" t="n">
-        <v>5545577128</v>
-      </c>
-      <c r="R174" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S174" s="50" t="inlineStr">
-        <is>
-          <t>COMPARTIDA</t>
-        </is>
-      </c>
-      <c r="T174" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="U174" s="50" t="n">
-        <v>22500</v>
-      </c>
-      <c r="V174" s="50" t="n">
-        <v>22500</v>
-      </c>
-      <c r="W174" s="35" t="inlineStr">
-        <is>
-          <t>Carranco 307 Residencial El Refugio, Querétaro 76146</t>
-        </is>
-      </c>
-      <c r="X174" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y174" s="50" t="n">
-        <v>5625</v>
-      </c>
-      <c r="Z174" s="50" t="inlineStr">
-        <is>
-          <t>CERRADA</t>
-        </is>
-      </c>
-      <c r="AA174" s="53" t="n">
-        <v>46224</v>
-      </c>
-      <c r="AB174" s="53" t="n">
-        <v>46232</v>
-      </c>
-      <c r="AC174" s="31" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AD174" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
+      <c r="C174" s="50" t="n"/>
+      <c r="D174" s="50" t="n"/>
+      <c r="E174" s="50" t="n"/>
+      <c r="F174" s="35" t="n"/>
+      <c r="G174" s="50" t="n"/>
+      <c r="H174" s="42" t="n"/>
+      <c r="I174" s="50" t="n"/>
+      <c r="J174" s="50" t="n"/>
+      <c r="K174" s="50" t="n"/>
+      <c r="L174" s="50" t="n"/>
+      <c r="M174" s="50" t="n"/>
+      <c r="N174" s="50" t="n"/>
+      <c r="O174" s="50" t="n"/>
+      <c r="P174" s="50" t="n"/>
+      <c r="Q174" s="50" t="n"/>
+      <c r="R174" s="50" t="n"/>
+      <c r="S174" s="50" t="n"/>
+      <c r="T174" s="51" t="n"/>
+      <c r="U174" s="50" t="n"/>
+      <c r="V174" s="50" t="n"/>
+      <c r="W174" s="35" t="n"/>
+      <c r="X174" s="50" t="n"/>
+      <c r="Y174" s="50" t="n"/>
+      <c r="Z174" s="50" t="n"/>
+      <c r="AA174" s="39" t="n"/>
+      <c r="AB174" s="39" t="n"/>
+      <c r="AC174" s="42" t="n"/>
+      <c r="AD174" s="50" t="n"/>
     </row>
     <row r="175" ht="22.5" customHeight="1" s="52">
-      <c r="A175" s="53" t="n"/>
+      <c r="A175" s="49" t="n"/>
       <c r="B175" s="50" t="n"/>
-      <c r="C175" s="50" t="n">
-        <v>6200</v>
-      </c>
-      <c r="D175" s="31" t="inlineStr">
-        <is>
-          <t>RENTA</t>
-        </is>
-      </c>
-      <c r="E175" s="50" t="inlineStr">
-        <is>
-          <t>TRANSFERENCIA</t>
-        </is>
-      </c>
-      <c r="F175" s="35" t="inlineStr">
-        <is>
-          <t>EB-WE5967</t>
-        </is>
-      </c>
-      <c r="G175" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="H175" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I175" s="50" t="inlineStr">
-        <is>
-          <t>Christian Díaz Padilla</t>
-        </is>
-      </c>
-      <c r="J175" s="50" t="inlineStr">
-        <is>
-          <t>Guardia</t>
-        </is>
-      </c>
-      <c r="K175" s="50" t="inlineStr">
-        <is>
-          <t>PAGADO</t>
-        </is>
-      </c>
-      <c r="L175" s="50" t="inlineStr">
-        <is>
-          <t>Mariana Vega Remax Terra</t>
-        </is>
-      </c>
-      <c r="M175" s="50" t="n">
-        <v>4424494148</v>
-      </c>
-      <c r="N175" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O175" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P175" s="50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mariana Brito de León </t>
-        </is>
-      </c>
-      <c r="Q175" s="50" t="inlineStr">
-        <is>
-          <t>‪55 5214 4405‬</t>
-        </is>
-      </c>
-      <c r="R175" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S175" s="50" t="inlineStr">
-        <is>
-          <t>COMPARTIDA</t>
-        </is>
-      </c>
-      <c r="T175" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="U175" s="50" t="n">
-        <v>6200</v>
-      </c>
-      <c r="V175" s="50" t="n">
-        <v>6200</v>
-      </c>
-      <c r="W175" s="35" t="inlineStr">
-        <is>
-          <t>Puertas de oyamel 131 22 Puertas de san Miguel, Querétaro</t>
-        </is>
-      </c>
-      <c r="X175" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y175" s="50" t="n">
-        <v>1550</v>
-      </c>
-      <c r="Z175" s="50" t="inlineStr">
-        <is>
-          <t>CERRADA</t>
-        </is>
-      </c>
-      <c r="AA175" s="53" t="n">
-        <v>46224</v>
-      </c>
-      <c r="AB175" s="53" t="n">
-        <v>46233</v>
-      </c>
-      <c r="AC175" s="31" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AD175" s="50" t="inlineStr">
-        <is>
-          <t>TRANSFERENCIA</t>
-        </is>
-      </c>
+      <c r="C175" s="50" t="n"/>
+      <c r="D175" s="50" t="n"/>
+      <c r="E175" s="50" t="n"/>
+      <c r="F175" s="35" t="n"/>
+      <c r="G175" s="50" t="n"/>
+      <c r="H175" s="42" t="n"/>
+      <c r="I175" s="50" t="n"/>
+      <c r="J175" s="50" t="n"/>
+      <c r="K175" s="50" t="n"/>
+      <c r="L175" s="50" t="n"/>
+      <c r="M175" s="50" t="n"/>
+      <c r="N175" s="50" t="n"/>
+      <c r="O175" s="50" t="n"/>
+      <c r="P175" s="50" t="n"/>
+      <c r="Q175" s="50" t="n"/>
+      <c r="R175" s="50" t="n"/>
+      <c r="S175" s="50" t="n"/>
+      <c r="T175" s="51" t="n"/>
+      <c r="U175" s="50" t="n"/>
+      <c r="V175" s="50" t="n"/>
+      <c r="W175" s="35" t="n"/>
+      <c r="X175" s="50" t="n"/>
+      <c r="Y175" s="50" t="n"/>
+      <c r="Z175" s="50" t="n"/>
+      <c r="AA175" s="39" t="n"/>
+      <c r="AB175" s="39" t="n"/>
+      <c r="AC175" s="42" t="n"/>
+      <c r="AD175" s="50" t="n"/>
     </row>
     <row r="176" ht="22.5" customHeight="1" s="52">
-      <c r="A176" s="53" t="n"/>
+      <c r="A176" s="49" t="n"/>
       <c r="B176" s="50" t="n"/>
-      <c r="C176" s="50" t="n">
-        <v>6170</v>
-      </c>
-      <c r="D176" s="31" t="inlineStr">
-        <is>
-          <t>RENTA</t>
-        </is>
-      </c>
-      <c r="E176" s="50" t="inlineStr">
-        <is>
-          <t>TRANSFERENCIA</t>
-        </is>
-      </c>
-      <c r="F176" s="35" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G176" s="50" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="H176" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I176" s="50" t="inlineStr">
-        <is>
-          <t>Christian Alvarado Martínez</t>
-        </is>
-      </c>
-      <c r="J176" s="50" t="inlineStr">
-        <is>
-          <t>Lona</t>
-        </is>
-      </c>
-      <c r="K176" s="50" t="inlineStr">
-        <is>
-          <t>PAGADO</t>
-        </is>
-      </c>
-      <c r="L176" s="50" t="inlineStr">
-        <is>
-          <t>María de los Ángeles Bostal Remax Terra</t>
-        </is>
-      </c>
-      <c r="M176" s="50" t="n">
-        <v>4428226699</v>
-      </c>
-      <c r="N176" s="50" t="inlineStr">
-        <is>
-          <t>Elias Maqueda</t>
-        </is>
-      </c>
-      <c r="O176" s="50" t="n">
-        <v>522941111423</v>
-      </c>
-      <c r="P176" s="50" t="inlineStr">
-        <is>
-          <t>Lizbeth Rodriguez</t>
-        </is>
-      </c>
-      <c r="Q176" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R176" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S176" s="50" t="inlineStr">
-        <is>
-          <t>COMPARTIDA</t>
-        </is>
-      </c>
-      <c r="T176" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="U176" s="50" t="n">
-        <v>6170</v>
-      </c>
-      <c r="V176" s="50" t="n">
-        <v>6170</v>
-      </c>
-      <c r="W176" s="35" t="inlineStr">
-        <is>
-          <t>Av. De las Fuentes 1502 11 Andadores Satélite, Qro Qro CP 76110</t>
-        </is>
-      </c>
-      <c r="X176" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y176" s="50" t="n">
-        <v>1542.5</v>
-      </c>
-      <c r="Z176" s="50" t="inlineStr">
-        <is>
-          <t>CERRADA</t>
-        </is>
-      </c>
-      <c r="AA176" s="53" t="n">
-        <v>46265</v>
-      </c>
-      <c r="AB176" s="53" t="n">
-        <v>46247</v>
-      </c>
-      <c r="AC176" s="31" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AD176" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
+      <c r="C176" s="50" t="n"/>
+      <c r="D176" s="50" t="n"/>
+      <c r="E176" s="50" t="n"/>
+      <c r="F176" s="35" t="n"/>
+      <c r="G176" s="50" t="n"/>
+      <c r="H176" s="42" t="n"/>
+      <c r="I176" s="50" t="n"/>
+      <c r="J176" s="50" t="n"/>
+      <c r="K176" s="50" t="n"/>
+      <c r="L176" s="50" t="n"/>
+      <c r="M176" s="50" t="n"/>
+      <c r="N176" s="50" t="n"/>
+      <c r="O176" s="50" t="n"/>
+      <c r="P176" s="50" t="n"/>
+      <c r="Q176" s="50" t="n"/>
+      <c r="R176" s="50" t="n"/>
+      <c r="S176" s="50" t="n"/>
+      <c r="T176" s="51" t="n"/>
+      <c r="U176" s="50" t="n"/>
+      <c r="V176" s="50" t="n"/>
+      <c r="W176" s="35" t="n"/>
+      <c r="X176" s="50" t="n"/>
+      <c r="Y176" s="50" t="n"/>
+      <c r="Z176" s="50" t="n"/>
+      <c r="AA176" s="39" t="n"/>
+      <c r="AB176" s="39" t="n"/>
+      <c r="AC176" s="42" t="n"/>
+      <c r="AD176" s="50" t="n"/>
     </row>
     <row r="177" ht="22.5" customHeight="1" s="52">
-      <c r="A177" s="53" t="n"/>
+      <c r="A177" s="49" t="n"/>
       <c r="B177" s="50" t="n"/>
-      <c r="C177" s="50" t="n">
-        <v>8000</v>
-      </c>
-      <c r="D177" s="31" t="inlineStr">
-        <is>
-          <t>RENTA</t>
-        </is>
-      </c>
-      <c r="E177" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
-      <c r="F177" s="35" t="inlineStr">
-        <is>
-          <t>CLR685373-495</t>
-        </is>
-      </c>
-      <c r="G177" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="H177" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I177" s="50" t="inlineStr">
-        <is>
-          <t>Adriana Regalado</t>
-        </is>
-      </c>
-      <c r="J177" s="50" t="inlineStr">
-        <is>
-          <t>Remax</t>
-        </is>
-      </c>
-      <c r="K177" s="50" t="inlineStr">
-        <is>
-          <t>PAGADO</t>
-        </is>
-      </c>
-      <c r="L177" s="50" t="inlineStr">
-        <is>
-          <t>María Elena Romano Pelayo Remax Terra</t>
-        </is>
-      </c>
-      <c r="M177" s="50" t="n">
-        <v>8711893807</v>
-      </c>
-      <c r="N177" s="50" t="inlineStr">
-        <is>
-          <t>Voluntarias Vicentinas de Querétaro AC</t>
-        </is>
-      </c>
-      <c r="O177" s="50" t="n">
-        <v>4411819918</v>
-      </c>
-      <c r="P177" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q177" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R177" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S177" s="50" t="inlineStr">
-        <is>
-          <t>COMPARTIDA</t>
-        </is>
-      </c>
-      <c r="T177" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="U177" s="50" t="n">
-        <v>8000</v>
-      </c>
-      <c r="V177" s="50" t="n">
-        <v>8000</v>
-      </c>
-      <c r="W177" s="35" t="inlineStr">
-        <is>
-          <t>Cuauhtémoc 5 Centro, Querétaro</t>
-        </is>
-      </c>
-      <c r="X177" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y177" s="50" t="n">
-        <v>2000</v>
-      </c>
-      <c r="Z177" s="50" t="inlineStr">
-        <is>
-          <t>CERRADA</t>
-        </is>
-      </c>
-      <c r="AA177" s="53" t="n">
-        <v>46244</v>
-      </c>
-      <c r="AB177" s="53" t="n">
-        <v>46266</v>
-      </c>
-      <c r="AC177" s="31" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AD177" s="50" t="inlineStr">
-        <is>
-          <t>EFECTIVO</t>
-        </is>
-      </c>
+      <c r="C177" s="50" t="n"/>
+      <c r="D177" s="50" t="n"/>
+      <c r="E177" s="50" t="n"/>
+      <c r="F177" s="35" t="n"/>
+      <c r="G177" s="50" t="n"/>
+      <c r="H177" s="42" t="n"/>
+      <c r="I177" s="50" t="n"/>
+      <c r="J177" s="50" t="n"/>
+      <c r="K177" s="50" t="n"/>
+      <c r="L177" s="50" t="n"/>
+      <c r="M177" s="50" t="n"/>
+      <c r="N177" s="50" t="n"/>
+      <c r="O177" s="50" t="n"/>
+      <c r="P177" s="50" t="n"/>
+      <c r="Q177" s="50" t="n"/>
+      <c r="R177" s="50" t="n"/>
+      <c r="S177" s="50" t="n"/>
+      <c r="T177" s="51" t="n"/>
+      <c r="U177" s="50" t="n"/>
+      <c r="V177" s="50" t="n"/>
+      <c r="W177" s="35" t="n"/>
+      <c r="X177" s="50" t="n"/>
+      <c r="Y177" s="50" t="n"/>
+      <c r="Z177" s="50" t="n"/>
+      <c r="AA177" s="39" t="n"/>
+      <c r="AB177" s="39" t="n"/>
+      <c r="AC177" s="42" t="n"/>
+      <c r="AD177" s="50" t="n"/>
     </row>
     <row r="178" ht="22.5" customHeight="1" s="52">
-      <c r="A178" s="53" t="n"/>
+      <c r="A178" s="49" t="n"/>
       <c r="B178" s="50" t="n"/>
-      <c r="C178" s="50" t="n">
-        <v>23000</v>
-      </c>
-      <c r="D178" s="31" t="inlineStr">
-        <is>
-          <t>RENTA</t>
-        </is>
-      </c>
-      <c r="E178" s="50" t="inlineStr">
-        <is>
-          <t>TRANSFERENCIA</t>
-        </is>
-      </c>
-      <c r="F178" s="35" t="inlineStr">
-        <is>
-          <t>RDR684910-495</t>
-        </is>
-      </c>
-      <c r="G178" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="H178" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I178" s="50" t="inlineStr">
-        <is>
-          <t>Adriana Calva</t>
-        </is>
-      </c>
-      <c r="J178" s="50" t="inlineStr">
-        <is>
-          <t>Recomendado</t>
-        </is>
-      </c>
-      <c r="K178" s="50" t="inlineStr">
-        <is>
-          <t>PAGADO</t>
-        </is>
-      </c>
-      <c r="L178" s="50" t="inlineStr">
-        <is>
-          <t>María Elena Romano Pelayo Remax Terra</t>
-        </is>
-      </c>
-      <c r="M178" s="50" t="n">
-        <v>5511287270</v>
-      </c>
-      <c r="N178" s="50" t="inlineStr">
-        <is>
-          <t>Vicentinas de Querpetaro AC</t>
-        </is>
-      </c>
-      <c r="O178" s="50" t="n">
-        <v>4411819918</v>
-      </c>
-      <c r="P178" s="50" t="inlineStr">
-        <is>
-          <t>Fernanda Acosta</t>
-        </is>
-      </c>
-      <c r="Q178" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R178" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S178" s="50" t="inlineStr">
-        <is>
-          <t>COMPARTIDA</t>
-        </is>
-      </c>
-      <c r="T178" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="U178" s="50" t="n">
-        <v>23000</v>
-      </c>
-      <c r="V178" s="50" t="n">
-        <v>23000</v>
-      </c>
-      <c r="W178" s="35" t="inlineStr">
-        <is>
-          <t>Cuauhtémoc No. 5 Col. Centro, Querétaro, Qro. 5 Centro, Querétaro</t>
-        </is>
-      </c>
-      <c r="X178" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y178" s="50" t="n">
-        <v>5750</v>
-      </c>
-      <c r="Z178" s="50" t="inlineStr">
-        <is>
-          <t>CERRADA</t>
-        </is>
-      </c>
-      <c r="AA178" s="53" t="n">
-        <v>46249</v>
-      </c>
-      <c r="AB178" s="53" t="n">
-        <v>46259</v>
-      </c>
-      <c r="AC178" s="31" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AD178" s="50" t="inlineStr">
-        <is>
-          <t>TRANSFERENCIA</t>
-        </is>
-      </c>
+      <c r="C178" s="50" t="n"/>
+      <c r="D178" s="50" t="n"/>
+      <c r="E178" s="50" t="n"/>
+      <c r="F178" s="35" t="n"/>
+      <c r="G178" s="50" t="n"/>
+      <c r="H178" s="42" t="n"/>
+      <c r="I178" s="50" t="n"/>
+      <c r="J178" s="50" t="n"/>
+      <c r="K178" s="50" t="n"/>
+      <c r="L178" s="50" t="n"/>
+      <c r="M178" s="50" t="n"/>
+      <c r="N178" s="50" t="n"/>
+      <c r="O178" s="50" t="n"/>
+      <c r="P178" s="50" t="n"/>
+      <c r="Q178" s="50" t="n"/>
+      <c r="R178" s="50" t="n"/>
+      <c r="S178" s="50" t="n"/>
+      <c r="T178" s="51" t="n"/>
+      <c r="U178" s="50" t="n"/>
+      <c r="V178" s="50" t="n"/>
+      <c r="W178" s="35" t="n"/>
+      <c r="X178" s="50" t="n"/>
+      <c r="Y178" s="50" t="n"/>
+      <c r="Z178" s="50" t="n"/>
+      <c r="AA178" s="39" t="n"/>
+      <c r="AB178" s="39" t="n"/>
+      <c r="AC178" s="42" t="n"/>
+      <c r="AD178" s="50" t="n"/>
     </row>
     <row r="179" ht="22.5" customHeight="1" s="52">
-      <c r="A179" s="53" t="n"/>
+      <c r="A179" s="49" t="n"/>
       <c r="B179" s="50" t="n"/>
-      <c r="C179" s="50" t="n">
-        <v>19000</v>
-      </c>
-      <c r="D179" s="31" t="inlineStr">
-        <is>
-          <t>RENTA</t>
-        </is>
-      </c>
-      <c r="E179" s="50" t="inlineStr">
-        <is>
-          <t>TRANSFERENCIA</t>
-        </is>
-      </c>
-      <c r="F179" s="35" t="inlineStr">
-        <is>
-          <t>RDR673241-495</t>
-        </is>
-      </c>
-      <c r="G179" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="H179" s="50" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I179" s="50" t="inlineStr">
-        <is>
-          <t>Pilar González Ávila</t>
-        </is>
-      </c>
-      <c r="J179" s="50" t="inlineStr">
-        <is>
-          <t>Inmuebles24</t>
-        </is>
-      </c>
-      <c r="K179" s="50" t="inlineStr">
-        <is>
-          <t>PAGADO</t>
-        </is>
-      </c>
-      <c r="L179" s="50" t="inlineStr">
-        <is>
-          <t>Erik Trotter Bustamante Remax Terra</t>
-        </is>
-      </c>
-      <c r="M179" s="50" t="n">
-        <v>4421814026</v>
-      </c>
-      <c r="N179" s="50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Daniela García Ramírez </t>
-        </is>
-      </c>
-      <c r="O179" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P179" s="50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Luis Miranda </t>
-        </is>
-      </c>
-      <c r="Q179" s="50" t="n">
-        <v>4425812243</v>
-      </c>
-      <c r="R179" s="50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S179" s="50" t="inlineStr">
-        <is>
-          <t>COMPARTIDA</t>
-        </is>
-      </c>
-      <c r="T179" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="U179" s="50" t="n">
-        <v>19000</v>
-      </c>
-      <c r="V179" s="50" t="n">
-        <v>19000</v>
-      </c>
-      <c r="W179" s="35" t="inlineStr">
-        <is>
-          <t>Ac constituyentes ote 40 apj 02 latitud la victoria 40 Apj 02 Villas del sol, Querétaro</t>
-        </is>
-      </c>
-      <c r="X179" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y179" s="50" t="n">
-        <v>7600</v>
-      </c>
-      <c r="Z179" s="50" t="inlineStr">
-        <is>
-          <t>CERRADA</t>
-        </is>
-      </c>
-      <c r="AA179" s="53" t="n">
-        <v>46267</v>
-      </c>
-      <c r="AB179" s="53" t="n">
-        <v>46268</v>
-      </c>
-      <c r="AC179" s="31" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AD179" s="50" t="inlineStr">
-        <is>
-          <t>TRANSFERENCIA</t>
-        </is>
-      </c>
+      <c r="C179" s="50" t="n"/>
+      <c r="D179" s="50" t="n"/>
+      <c r="E179" s="50" t="n"/>
+      <c r="F179" s="35" t="n"/>
+      <c r="G179" s="50" t="n"/>
+      <c r="H179" s="42" t="n"/>
+      <c r="I179" s="50" t="n"/>
+      <c r="J179" s="50" t="n"/>
+      <c r="K179" s="50" t="n"/>
+      <c r="L179" s="50" t="n"/>
+      <c r="M179" s="50" t="n"/>
+      <c r="N179" s="50" t="n"/>
+      <c r="O179" s="50" t="n"/>
+      <c r="P179" s="50" t="n"/>
+      <c r="Q179" s="50" t="n"/>
+      <c r="R179" s="50" t="n"/>
+      <c r="S179" s="50" t="n"/>
+      <c r="T179" s="51" t="n"/>
+      <c r="U179" s="50" t="n"/>
+      <c r="V179" s="50" t="n"/>
+      <c r="W179" s="35" t="n"/>
+      <c r="X179" s="50" t="n"/>
+      <c r="Y179" s="50" t="n"/>
+      <c r="Z179" s="50" t="n"/>
+      <c r="AA179" s="39" t="n"/>
+      <c r="AB179" s="39" t="n"/>
+      <c r="AC179" s="42" t="n"/>
+      <c r="AD179" s="50" t="n"/>
     </row>
     <row r="180" ht="22.5" customHeight="1" s="52">
       <c r="A180" s="49" t="n"/>

</xml_diff>